<commit_message>
added lie_group formulation without classes
</commit_message>
<xml_diff>
--- a/ra/time data (version 2).xlsb.xlsx
+++ b/ra/time data (version 2).xlsb.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\uni\masters nu\RA\pythonCode\ra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF410155-A0C0-4D11-A342-5FEAD89CA603}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9101D87-BA3A-434D-86D6-F4C78D1A24C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2231,6 +2231,102 @@
             </c:ext>
           </c:extLst>
         </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'5s 500'!$I$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Log GA</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>'5s 500'!$I$2:$I$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>-0.79377661948310396</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.76661370790106853</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-0.66861056674877373</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.58215230249782446</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.49799563519949192</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-0.4140330767873921</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.37394206723934081</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.32377915989853379</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-0.29307791681275264</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-0.25194383246322088</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-0.21196087548954762</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-0.16804849135734951</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-0.15033162931084057</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-0.12076788696980725</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-7.5895966342748949E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-6.9049594150897398E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-3.3840285499332941E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-2.1050763898457017E-2</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>9.3525522273099487E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-245C-462D-8B8A-37780AC87CF8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
@@ -2481,8 +2577,8 @@
           <c:yMode val="edge"/>
           <c:x val="0.13053999828968746"/>
           <c:y val="0.11762405856546715"/>
-          <c:w val="0.10201027786493486"/>
-          <c:h val="0.1965019209542527"/>
+          <c:w val="6.6754456035186593E-2"/>
+          <c:h val="0.20497131901064805"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -15800,19 +15896,19 @@
         <v>0.171153699979186</v>
       </c>
       <c r="F3">
-        <f>LOG(B3)</f>
+        <f t="shared" ref="F3:F20" si="0">LOG(B3)</f>
         <v>-0.41184038361690795</v>
       </c>
       <c r="G3">
-        <f>LOG(C3)</f>
+        <f t="shared" ref="G3:G20" si="1">LOG(C3)</f>
         <v>0.36310406607463558</v>
       </c>
       <c r="H3">
-        <f>LOG(D3)</f>
+        <f t="shared" ref="H3:H20" si="2">LOG(D3)</f>
         <v>-0.90413354652145739</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I20" si="0">LOG(E3)</f>
+        <f t="shared" ref="I3:I20" si="3">LOG(E3)</f>
         <v>-0.76661370790106853</v>
       </c>
     </row>
@@ -15833,19 +15929,19 @@
         <v>0.214481299975886</v>
       </c>
       <c r="F4">
-        <f>LOG(B4)</f>
+        <f t="shared" si="0"/>
         <v>-0.2438966284148944</v>
       </c>
       <c r="G4">
-        <f>LOG(C4)</f>
+        <f t="shared" si="1"/>
         <v>0.89795131674577622</v>
       </c>
       <c r="H4">
-        <f>LOG(D4)</f>
+        <f t="shared" si="2"/>
         <v>-0.77754366332075331</v>
       </c>
       <c r="I4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.66861056674877373</v>
       </c>
     </row>
@@ -15866,19 +15962,19 @@
         <v>0.261726500000804</v>
       </c>
       <c r="F5">
-        <f>LOG(B5)</f>
+        <f t="shared" si="0"/>
         <v>-0.18217030025439443</v>
       </c>
       <c r="G5">
-        <f>LOG(C5)</f>
+        <f t="shared" si="1"/>
         <v>1.2963492248187813</v>
       </c>
       <c r="H5">
-        <f>LOG(D5)</f>
+        <f t="shared" si="2"/>
         <v>-0.64416550411506401</v>
       </c>
       <c r="I5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.58215230249782446</v>
       </c>
     </row>
@@ -15899,19 +15995,19 @@
         <v>0.31769059994257898</v>
       </c>
       <c r="F6">
-        <f>LOG(B6)</f>
+        <f t="shared" si="0"/>
         <v>3.4106829707643734E-2</v>
       </c>
       <c r="G6">
-        <f>LOG(C6)</f>
+        <f t="shared" si="1"/>
         <v>1.635410352888679</v>
       </c>
       <c r="H6">
-        <f>LOG(D6)</f>
+        <f t="shared" si="2"/>
         <v>-0.44903824770182388</v>
       </c>
       <c r="I6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.49799563519949192</v>
       </c>
     </row>
@@ -15932,19 +16028,19 @@
         <v>0.38544899993576098</v>
       </c>
       <c r="F7">
-        <f>LOG(B7)</f>
+        <f t="shared" si="0"/>
         <v>6.8482713761754369E-2</v>
       </c>
       <c r="G7">
-        <f>LOG(C7)</f>
+        <f t="shared" si="1"/>
         <v>1.9054812401049357</v>
       </c>
       <c r="H7">
-        <f>LOG(D7)</f>
+        <f t="shared" si="2"/>
         <v>-0.41998788747057569</v>
       </c>
       <c r="I7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.4140330767873921</v>
       </c>
     </row>
@@ -15965,19 +16061,19 @@
         <v>0.42272499995306101</v>
       </c>
       <c r="F8">
-        <f>LOG(B8)</f>
+        <f t="shared" si="0"/>
         <v>0.13110516209373138</v>
       </c>
       <c r="G8">
-        <f>LOG(C8)</f>
+        <f t="shared" si="1"/>
         <v>2.1588402547316026</v>
       </c>
       <c r="H8">
-        <f>LOG(D8)</f>
+        <f t="shared" si="2"/>
         <v>-0.39968067024833892</v>
       </c>
       <c r="I8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.37394206723934081</v>
       </c>
     </row>
@@ -15998,19 +16094,19 @@
         <v>0.47448320011608303</v>
       </c>
       <c r="F9">
-        <f>LOG(B9)</f>
+        <f t="shared" si="0"/>
         <v>0.21351775699630487</v>
       </c>
       <c r="G9">
-        <f>LOG(C9)</f>
+        <f t="shared" si="1"/>
         <v>2.3972014278122304</v>
       </c>
       <c r="H9">
-        <f>LOG(D9)</f>
+        <f t="shared" si="2"/>
         <v>-0.35595550718525121</v>
       </c>
       <c r="I9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.32377915989853379</v>
       </c>
     </row>
@@ -16031,19 +16127,19 @@
         <v>0.50923950015567199</v>
       </c>
       <c r="F10">
-        <f>LOG(B10)</f>
+        <f t="shared" si="0"/>
         <v>0.24968742780530151</v>
       </c>
       <c r="G10">
-        <f>LOG(C10)</f>
+        <f t="shared" si="1"/>
         <v>2.5560865061967952</v>
       </c>
       <c r="H10">
-        <f>LOG(D10)</f>
+        <f t="shared" si="2"/>
         <v>-0.26640153903866087</v>
       </c>
       <c r="I10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.29307791681275264</v>
       </c>
     </row>
@@ -16064,19 +16160,19 @@
         <v>0.55982999992556803</v>
       </c>
       <c r="F11">
-        <f>LOG(B11)</f>
+        <f t="shared" si="0"/>
         <v>0.27664559363087632</v>
       </c>
       <c r="G11">
-        <f>LOG(C11)</f>
+        <f t="shared" si="1"/>
         <v>2.7808634738027793</v>
       </c>
       <c r="H11">
-        <f>LOG(D11)</f>
+        <f t="shared" si="2"/>
         <v>-0.31722335368556592</v>
       </c>
       <c r="I11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.25194383246322088</v>
       </c>
     </row>
@@ -16097,19 +16193,19 @@
         <v>0.61381729994900502</v>
       </c>
       <c r="F12">
-        <f>LOG(B12)</f>
+        <f t="shared" si="0"/>
         <v>0.3280124388555864</v>
       </c>
       <c r="G12">
-        <f>LOG(C12)</f>
+        <f t="shared" si="1"/>
         <v>2.9578717096022213</v>
       </c>
       <c r="H12">
-        <f>LOG(D12)</f>
+        <f t="shared" si="2"/>
         <v>-0.21218543293697692</v>
       </c>
       <c r="I12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.21196087548954762</v>
       </c>
     </row>
@@ -16130,19 +16226,19 @@
         <v>0.67912780004553497</v>
       </c>
       <c r="F13">
-        <f>LOG(B13)</f>
+        <f t="shared" si="0"/>
         <v>0.3802293369380374</v>
       </c>
       <c r="G13">
-        <f>LOG(C13)</f>
+        <f t="shared" si="1"/>
         <v>3.0642572313915459</v>
       </c>
       <c r="H13">
-        <f>LOG(D13)</f>
+        <f t="shared" si="2"/>
         <v>-0.21645371772965016</v>
       </c>
       <c r="I13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.16804849135734951</v>
       </c>
     </row>
@@ -16163,19 +16259,19 @@
         <v>0.70740539999678698</v>
       </c>
       <c r="F14">
-        <f>LOG(B14)</f>
+        <f t="shared" si="0"/>
         <v>0.34161255871200186</v>
       </c>
       <c r="G14">
-        <f>LOG(C14)</f>
+        <f t="shared" si="1"/>
         <v>3.3825190202340627</v>
       </c>
       <c r="H14">
-        <f>LOG(D14)</f>
+        <f t="shared" si="2"/>
         <v>-0.19681611146465802</v>
       </c>
       <c r="I14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.15033162931084057</v>
       </c>
     </row>
@@ -16196,19 +16292,19 @@
         <v>0.75723750004544799</v>
       </c>
       <c r="F15">
-        <f>LOG(B15)</f>
+        <f t="shared" si="0"/>
         <v>0.40898576821169425</v>
       </c>
       <c r="G15">
-        <f>LOG(C15)</f>
+        <f t="shared" si="1"/>
         <v>3.3818388011015577</v>
       </c>
       <c r="H15">
-        <f>LOG(D15)</f>
+        <f t="shared" si="2"/>
         <v>1.8866863150906826E-2</v>
       </c>
       <c r="I15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.12076788696980725</v>
       </c>
     </row>
@@ -16229,19 +16325,19 @@
         <v>0.83966110018081896</v>
       </c>
       <c r="F16">
-        <f>LOG(B16)</f>
+        <f t="shared" si="0"/>
         <v>0.44805671088621207</v>
       </c>
       <c r="G16">
-        <f>LOG(C16)</f>
+        <f t="shared" si="1"/>
         <v>3.5141481507647532</v>
       </c>
       <c r="H16">
-        <f>LOG(D16)</f>
+        <f t="shared" si="2"/>
         <v>-7.8001568691729029E-2</v>
       </c>
       <c r="I16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-7.5895966342748949E-2</v>
       </c>
     </row>
@@ -16262,19 +16358,19 @@
         <v>0.85300270002335299</v>
       </c>
       <c r="F17">
-        <f>LOG(B17)</f>
+        <f t="shared" si="0"/>
         <v>0.41308172370882884</v>
       </c>
       <c r="G17">
-        <f>LOG(C17)</f>
+        <f t="shared" si="1"/>
         <v>3.6022549457863358</v>
       </c>
       <c r="H17">
-        <f>LOG(D17)</f>
+        <f t="shared" si="2"/>
         <v>-0.12355121312165876</v>
       </c>
       <c r="I17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-6.9049594150897398E-2</v>
       </c>
     </row>
@@ -16295,19 +16391,19 @@
         <v>0.92503829998895504</v>
       </c>
       <c r="F18">
-        <f>LOG(B18)</f>
+        <f t="shared" si="0"/>
         <v>0.44745263122699308</v>
       </c>
       <c r="G18">
-        <f>LOG(C18)</f>
+        <f t="shared" si="1"/>
         <v>3.7558622660472802</v>
       </c>
       <c r="H18">
-        <f>LOG(D18)</f>
+        <f t="shared" si="2"/>
         <v>-9.2481153893370735E-2</v>
       </c>
       <c r="I18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-3.3840285499332941E-2</v>
       </c>
     </row>
@@ -16328,19 +16424,19 @@
         <v>0.95268479990772903</v>
       </c>
       <c r="F19">
-        <f>LOG(B19)</f>
+        <f t="shared" si="0"/>
         <v>0.48208714182648593</v>
       </c>
       <c r="G19">
-        <f>LOG(C19)</f>
+        <f t="shared" si="1"/>
         <v>3.8363828841125054</v>
       </c>
       <c r="H19">
-        <f>LOG(D19)</f>
+        <f t="shared" si="2"/>
         <v>-8.4178212379601269E-2</v>
       </c>
       <c r="I19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-2.1050763898457017E-2</v>
       </c>
     </row>
@@ -16361,19 +16457,19 @@
         <v>1.0217685999814401</v>
       </c>
       <c r="F20">
-        <f>LOG(B20)</f>
+        <f t="shared" si="0"/>
         <v>0.52937901628761841</v>
       </c>
       <c r="G20">
-        <f>LOG(C20)</f>
+        <f t="shared" si="1"/>
         <v>3.8922811035562344</v>
       </c>
       <c r="H20">
-        <f>LOG(D20)</f>
+        <f t="shared" si="2"/>
         <v>-6.5905731644519627E-2</v>
       </c>
       <c r="I20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>9.3525522273099487E-3</v>
       </c>
     </row>
@@ -16472,19 +16568,19 @@
         <v>0.34577620006166399</v>
       </c>
       <c r="F3">
-        <f>LOG(B3)</f>
+        <f t="shared" ref="F3:F20" si="0">LOG(B3)</f>
         <v>-0.11599807523121287</v>
       </c>
       <c r="G3">
-        <f>LOG(C3)</f>
+        <f t="shared" ref="G3:G20" si="1">LOG(C3)</f>
         <v>0.67105244589460922</v>
       </c>
       <c r="H3">
-        <f>LOG(D3)</f>
+        <f t="shared" ref="H3:H20" si="2">LOG(D3)</f>
         <v>-0.59209945985736478</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I20" si="0">LOG(E3)</f>
+        <f t="shared" ref="I3:I20" si="3">LOG(E3)</f>
         <v>-0.46120490272665071</v>
       </c>
     </row>
@@ -16505,19 +16601,19 @@
         <v>0.45446829986758502</v>
       </c>
       <c r="F4">
-        <f>LOG(B4)</f>
+        <f t="shared" si="0"/>
         <v>1.7617573339673596E-2</v>
       </c>
       <c r="G4">
-        <f>LOG(C4)</f>
+        <f t="shared" si="1"/>
         <v>1.1409100977860087</v>
       </c>
       <c r="H4">
-        <f>LOG(D4)</f>
+        <f t="shared" si="2"/>
         <v>-0.45917018588892017</v>
       </c>
       <c r="I4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.34249640435118378</v>
       </c>
     </row>
@@ -16538,19 +16634,19 @@
         <v>0.56685939989984002</v>
       </c>
       <c r="F5">
-        <f>LOG(B5)</f>
+        <f t="shared" si="0"/>
         <v>0.12531857812352648</v>
       </c>
       <c r="G5">
-        <f>LOG(C5)</f>
+        <f t="shared" si="1"/>
         <v>1.5271966790930642</v>
       </c>
       <c r="H5">
-        <f>LOG(D5)</f>
+        <f t="shared" si="2"/>
         <v>-0.37986394502624249</v>
       </c>
       <c r="I5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.24652464731471119</v>
       </c>
     </row>
@@ -16571,19 +16667,19 @@
         <v>0.66382870008237604</v>
       </c>
       <c r="F6">
-        <f>LOG(B6)</f>
+        <f t="shared" si="0"/>
         <v>0.20319612493503247</v>
       </c>
       <c r="G6">
-        <f>LOG(C6)</f>
+        <f t="shared" si="1"/>
         <v>1.8585053160566041</v>
       </c>
       <c r="H6">
-        <f>LOG(D6)</f>
+        <f t="shared" si="2"/>
         <v>-0.29782804914228878</v>
       </c>
       <c r="I6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.17794397516037561</v>
       </c>
     </row>
@@ -16604,19 +16700,19 @@
         <v>0.77235410013236105</v>
       </c>
       <c r="F7">
-        <f>LOG(B7)</f>
+        <f t="shared" si="0"/>
         <v>0.27535743108759814</v>
       </c>
       <c r="G7">
-        <f>LOG(C7)</f>
+        <f t="shared" si="1"/>
         <v>2.1812606136527593</v>
       </c>
       <c r="H7">
-        <f>LOG(D7)</f>
+        <f t="shared" si="2"/>
         <v>-0.22966355890485077</v>
       </c>
       <c r="I7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-0.11218354360775146</v>
       </c>
     </row>
@@ -16637,19 +16733,19 @@
         <v>0.9346729000099</v>
       </c>
       <c r="F8">
-        <f>LOG(B8)</f>
+        <f t="shared" si="0"/>
         <v>0.34543254749914665</v>
       </c>
       <c r="G8">
-        <f>LOG(C8)</f>
+        <f t="shared" si="1"/>
         <v>2.4659724668498528</v>
       </c>
       <c r="H8">
-        <f>LOG(D8)</f>
+        <f t="shared" si="2"/>
         <v>-0.14182386201765568</v>
       </c>
       <c r="I8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>-2.9340349100993781E-2</v>
       </c>
     </row>
@@ -16670,19 +16766,19 @@
         <v>1.03519709990359</v>
       </c>
       <c r="F9">
-        <f>LOG(B9)</f>
+        <f t="shared" si="0"/>
         <v>0.40418349821266247</v>
       </c>
       <c r="G9">
-        <f>LOG(C9)</f>
+        <f t="shared" si="1"/>
         <v>2.6833771387458261</v>
       </c>
       <c r="H9">
-        <f>LOG(D9)</f>
+        <f t="shared" si="2"/>
         <v>-0.10623823794205658</v>
       </c>
       <c r="I9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1.5023046653805916E-2</v>
       </c>
     </row>
@@ -16703,19 +16799,19 @@
         <v>1.08264300017617</v>
       </c>
       <c r="F10">
-        <f>LOG(B10)</f>
+        <f t="shared" si="0"/>
         <v>0.44966349415333057</v>
       </c>
       <c r="G10">
-        <f>LOG(C10)</f>
+        <f t="shared" si="1"/>
         <v>2.8452488381001197</v>
       </c>
       <c r="H10">
-        <f>LOG(D10)</f>
+        <f t="shared" si="2"/>
         <v>-6.7678468010706816E-2</v>
       </c>
       <c r="I10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>3.4485272310157057E-2</v>
       </c>
     </row>
@@ -16736,19 +16832,19 @@
         <v>1.25342390011064</v>
       </c>
       <c r="F11">
-        <f>LOG(B11)</f>
+        <f t="shared" si="0"/>
         <v>0.49590494359435922</v>
       </c>
       <c r="G11">
-        <f>LOG(C11)</f>
+        <f t="shared" si="1"/>
         <v>3.10556372742424</v>
       </c>
       <c r="H11">
-        <f>LOG(D11)</f>
+        <f t="shared" si="2"/>
         <v>-1.7050711425501325E-2</v>
       </c>
       <c r="I11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>9.8097971509004067E-2</v>
       </c>
     </row>
@@ -16769,19 +16865,19 @@
         <v>1.3160284000914499</v>
       </c>
       <c r="F12">
-        <f>LOG(B12)</f>
+        <f t="shared" si="0"/>
         <v>0.54841398855423695</v>
       </c>
       <c r="G12">
-        <f>LOG(C12)</f>
+        <f t="shared" si="1"/>
         <v>3.2405537659200929</v>
       </c>
       <c r="H12">
-        <f>LOG(D12)</f>
+        <f t="shared" si="2"/>
         <v>1.5401673702949125E-2</v>
       </c>
       <c r="I12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.11926526151951455</v>
       </c>
     </row>
@@ -16802,19 +16898,19 @@
         <v>1.4285178000573</v>
       </c>
       <c r="F13">
-        <f>LOG(B13)</f>
+        <f t="shared" si="0"/>
         <v>0.582608730687733</v>
       </c>
       <c r="G13">
-        <f>LOG(C13)</f>
+        <f t="shared" si="1"/>
         <v>3.406771963700217</v>
       </c>
       <c r="H13">
-        <f>LOG(D13)</f>
+        <f t="shared" si="2"/>
         <v>6.3633545230784669E-2</v>
       </c>
       <c r="I13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.15488565628228998</v>
       </c>
     </row>
@@ -16835,19 +16931,19 @@
         <v>1.50050369999371</v>
       </c>
       <c r="F14">
-        <f>LOG(B14)</f>
+        <f t="shared" si="0"/>
         <v>0.62727366165808607</v>
       </c>
       <c r="G14">
-        <f>LOG(C14)</f>
+        <f t="shared" si="1"/>
         <v>3.5277273291284281</v>
       </c>
       <c r="H14">
-        <f>LOG(D14)</f>
+        <f t="shared" si="2"/>
         <v>9.2580300691311124E-2</v>
       </c>
       <c r="I14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.17623707066048502</v>
       </c>
     </row>
@@ -16868,19 +16964,19 @@
         <v>1.6809717998839899</v>
       </c>
       <c r="F15">
-        <f>LOG(B15)</f>
+        <f t="shared" si="0"/>
         <v>0.6592504687726608</v>
       </c>
       <c r="G15">
-        <f>LOG(C15)</f>
+        <f t="shared" si="1"/>
         <v>3.6850515935762131</v>
       </c>
       <c r="H15">
-        <f>LOG(D15)</f>
+        <f t="shared" si="2"/>
         <v>0.11347539853673715</v>
       </c>
       <c r="I15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.22556042774196874</v>
       </c>
     </row>
@@ -16901,19 +16997,19 @@
         <v>1.73551960010081</v>
       </c>
       <c r="F16">
-        <f>LOG(B16)</f>
+        <f t="shared" si="0"/>
         <v>0.68306505838291154</v>
       </c>
       <c r="G16">
-        <f>LOG(C16)</f>
+        <f t="shared" si="1"/>
         <v>3.925712216048606</v>
       </c>
       <c r="H16">
-        <f>LOG(D16)</f>
+        <f t="shared" si="2"/>
         <v>0.15048012227033458</v>
       </c>
       <c r="I16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.23942952274241205</v>
       </c>
     </row>
@@ -16934,19 +17030,19 @@
         <v>1.8310300000011901</v>
       </c>
       <c r="F17">
-        <f>LOG(B17)</f>
+        <f t="shared" si="0"/>
         <v>0.72226362737262384</v>
       </c>
       <c r="G17">
-        <f>LOG(C17)</f>
+        <f t="shared" si="1"/>
         <v>4.0496315590090868</v>
       </c>
       <c r="H17">
-        <f>LOG(D17)</f>
+        <f t="shared" si="2"/>
         <v>0.17808443287921172</v>
       </c>
       <c r="I17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.26269545993699944</v>
       </c>
     </row>
@@ -16967,19 +17063,19 @@
         <v>1.9423700999468501</v>
       </c>
       <c r="F18">
-        <f>LOG(B18)</f>
+        <f t="shared" si="0"/>
         <v>0.75321524647887972</v>
       </c>
       <c r="G18">
-        <f>LOG(C18)</f>
+        <f t="shared" si="1"/>
         <v>4.1651177174029792</v>
       </c>
       <c r="H18">
-        <f>LOG(D18)</f>
+        <f t="shared" si="2"/>
         <v>0.19816203904607557</v>
       </c>
       <c r="I18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.28833198409448535</v>
       </c>
     </row>
@@ -17000,19 +17096,19 @@
         <v>2.0479162000119602</v>
       </c>
       <c r="F19">
-        <f>LOG(B19)</f>
+        <f t="shared" si="0"/>
         <v>0.78015162924532189</v>
       </c>
       <c r="G19">
-        <f>LOG(C19)</f>
+        <f t="shared" si="1"/>
         <v>4.2150346747474483</v>
       </c>
       <c r="H19">
-        <f>LOG(D19)</f>
+        <f t="shared" si="2"/>
         <v>0.22549020007128417</v>
       </c>
       <c r="I19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.31131218149471546</v>
       </c>
     </row>
@@ -17033,19 +17129,19 @@
         <v>2.2034616000019001</v>
       </c>
       <c r="F20">
-        <f>LOG(B20)</f>
+        <f t="shared" si="0"/>
         <v>0.80154090619031826</v>
       </c>
       <c r="G20">
-        <f>LOG(C20)</f>
+        <f t="shared" si="1"/>
         <v>4.249645026330171</v>
       </c>
       <c r="H20">
-        <f>LOG(D20)</f>
+        <f t="shared" si="2"/>
         <v>0.24487062206524232</v>
       </c>
       <c r="I20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.34310548640818223</v>
       </c>
     </row>

</xml_diff>